<commit_message>
Apply catalog batch (rename + refresh dashboard)
</commit_message>
<xml_diff>
--- a/docs/knowledge_chest.xlsx
+++ b/docs/knowledge_chest.xlsx
@@ -11,8 +11,8 @@
     <sheet name="Dataset Universe" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Papers'!$A$1:$L$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Dataset Universe'!$A$1:$I$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Papers'!$A$1:$L$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Dataset Universe'!$A$1:$I$45</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -518,7 +518,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Working Paper - 2026 - Correia et al. - Bank Runs with and without Bank Failure</t>
+          <t>Working Paper - 2026 - Egan et al. - Who Pays for Payments</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -527,50 +527,50 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Correia, Luck, Verner</t>
+          <t>Egan, Matvos, Seru, Wang, Yao</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Bank Runs with and without Bank Failure</t>
+          <t>Who Pays for Payments?</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>This paper builds a comprehensive historical database of U.S. bank runs by applying large language models to historical newspapers, yielding information on 3,984 runs on individual banks from 1863 to 1934. The data show runs are far more likely at weak banks but also occur at strong banks, especially following negative news about the real economy or the broader banking system. Crucially, runs typically cause failure only when a bank's fundamentals are poor; strong banks survive through signaling, interbank cooperation, and temporary suspension. Locally, runs on weak banks produce much larger declines in deposits, lending, and manufacturing activity than runs on strong banks. The findings put poor fundamentals at the center of both when runs occur and when they are economically damaging, tempering pure self-fulfilling-panic accounts.</t>
+          <t>This paper uses novel data on the composition and cost of payments across U.S. merchants to quantify redistribution in the payment system. Card interchange fees fund consumer rewards, and when merchants raise prices for everyone, users of low-cost methods like cash and debit cross-subsidize high-reward credit-card users at the same merchant. The authors show incidence actually depends on the joint distribution of payment choices across merchants, not the standard assumption that everyone shops at the same stores facing the same fees. Two forces shape redistribution: consumer sorting, where users of different payment methods shop at different merchants, limits cash and debit users' exposure to high interchange fees; and interchange fees vary across merchants, being lower where payment types overlap (e.g., large grocery stores) due to sector discounts and negotiations. Embedding these forces in a sufficient-statistics framework, the paper revises who ultimately bears payment-system costs.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>The paper's first contribution is measurement: it uses LLMs to read historical newspapers and assemble a large, bank-level database of runs spanning 1863-1934. With this data, it asks whether runs strike indiscriminately or track fundamentals, showing runs concentrate in weak banks yet can hit strong banks after adverse news. It then distinguishes runs from failures, documenting that strong banks survive runs via signaling, cooperation, and suspension, so that failure requires poor fundamentals. Finally it links runs to local real outcomes, showing damage is concentrated where fundamentals are weak, which it interprets as evidence against models where small shocks trigger discontinuous jumps to bad equilibria.</t>
+          <t>The paper reconsiders the common claim that low-reward payers subsidize high-reward card users, noting it assumes uniform shopping and fees. Using merchant-level payment data, it documents two overlooked forces - consumer sorting across merchants and cross-merchant variation in interchange fees. It shows sorting insulates cash and debit users from high-fee exposure, while fee variation further shapes overlap points. It then embeds these forces in a sufficient-statistics incidence framework to recompute the direction and magnitude of cross-subsidies in the payment system.</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Construction of a novel bank-level historical dataset via large language models applied to newspaper archives, combined with empirical analysis relating runs to bank fundamentals, survival mechanisms, and local real-economy outcomes.</t>
+          <t>A sufficient-statistics incidence framework estimated on proprietary merchant-acquirer payment data, combined with consumer payment-diary data, to quantify cross-subsidies under consumer sorting and merchant-level fee variation.</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Banking History, Financial Crises, Text-as-Data / LLMs</t>
+          <t>Payments, Household Finance, Industrial Organization</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Correia, Luck &amp; Verner (this paper) — Historical bank-run database; Library of Congress — Chronicling America; OCC — National bank call reports (Annual Report to Congress)</t>
+          <t>Fiserv; Federal Reserve Bank of Atlanta — Diary of Consumer Payment Choice (DCPC); Nilson Report</t>
         </is>
       </c>
       <c r="K2" s="2" t="n"/>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>/home/runner/work/Knowledge-Chest/Knowledge-Chest/Working Paper - 2026 - Correia et al. - Bank Runs with and without Bank Failure.pdf</t>
+          <t>/home/runner/work/Knowledge-Chest/Knowledge-Chest/Working Paper - 2026 - Egan et al. - Who Pays for Payments.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Working Paper - 2026 - Bornstein and Castillo-Martinez - Firm Exit and Financial Frictions</t>
+          <t>Working Paper - 2026 - Drechsler et al. - Credit Crunches and the Great Stagflation</t>
         </is>
       </c>
       <c r="B3" s="2" t="n"/>
@@ -579,50 +579,50 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Bornstein, Castillo-Martinez</t>
+          <t>Drechsler, Savov, Schnabl</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Firm Exit and Financial Frictions</t>
+          <t>Credit Crunches and the Great Stagflation</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>This paper examines whether financial frictions cause too many firms to fail, motivating government interventions that prevent closures during crises. The authors build a firm-dynamics model with incomplete financial markets and show that frictions generate excessive firm exit, with a key sufficient statistic being the marginal propensity to exit with debt. Using confidential U.S. Census data, they estimate the debt–exit relationship and use it to discipline the model. The calibrated model implies that eliminating financial frictions would cut firm exit from 9.3% to 5.0% and deliver welfare gains of 3.6% in consumption-equivalent terms, with costs that spike during financial crises but not during ordinary productivity recessions. Comparing government-guaranteed loans and grants, the paper quantifies the trade-off between fiscal cost and effectiveness in preventing excessive exit.</t>
+          <t>This paper argues that severe banking-system credit crunches helped cause the Great Stagflation of the 1970s, working through Regulation Q, which capped deposit rates. Under Reg Q, Fed tightening triggered large deposit outflows that forced banks to contract lending, and these credit crunches line up closely with stagflation over time. Adding Reg Q to a standard model where firms finance working capital with bank loans, the authors show binding caps make working capital costlier, leading firms to raise prices and cut output. This yields an augmented Phillips curve in which monetary tightening reduces aggregate supply as well as demand, with effects increasing in credit-crunch severity, external-finance dependence, and working-capital intensity. Cross-industry tests confirm that more exposed manufacturing industries raised prices and cut output relative to others.</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>The paper starts from the policy fear that viable-but-constrained firms fail in crises, and asks when firm exit is actually inefficient. It develops a firm-dynamics model with incomplete markets in which financial frictions distort the exit margin, isolating the marginal propensity to exit with debt as the statistic governing dynamic inefficiency. It then estimates the debt–exit relationship in confidential Census data to discipline that statistic and calibrate the model. Using the calibrated model, it quantifies the welfare cost of frictions across crisis and non-crisis states and evaluates guaranteed loans versus grants as interventions.</t>
+          <t>The paper links a monetary-institutional feature - Regulation Q deposit-rate caps - to the macro puzzle of simultaneous high inflation and stagnation. It explains how Fed tightening under Reg Q caused deposit outflows and lending contractions, then documents that these credit crunches track stagflation in the time series. It embeds Reg Q in a working-capital model, deriving an augmented Phillips curve where tighter credit raises firms' costs and shifts aggregate supply inward. It then tests the model's cross-sectional predictions across manufacturing industries by exposure, external-finance dependence, and working-capital intensity.</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>A quantitative firm-dynamics model with incomplete financial markets, disciplined by a reduced-form debt–exit relationship estimated on confidential U.S. Census microdata, used for welfare analysis and policy (loan-guarantee vs. grant) comparison.</t>
+          <t>A quantitative macro model (working-capital channel with Regulation Q) combined with time-series evidence and cross-industry exposure-based empirical tests of its supply-side predictions.</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>Firm Dynamics, Financial Frictions, Macroeconomic Policy</t>
+          <t>Monetary Economics, Banking, Macro-Finance</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>U.S. Census Bureau — Longitudinal Business Database (LBD); Bureau van Dijk — Orbis (Italy)</t>
+          <t>U.S. Call Reports (via FOIA); NBER-CES — Manufacturing Industry Database; FDIC — Historical Bank Data; Federal Reserve — Senior Loan Officer Opinion Survey (SLOOS)</t>
         </is>
       </c>
       <c r="K3" s="2" t="n"/>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>/home/runner/work/Knowledge-Chest/Knowledge-Chest/Working Paper - 2026 - Bornstein and Castillo-Martinez - Firm Exit and Financial Frictions.pdf</t>
+          <t>/home/runner/work/Knowledge-Chest/Knowledge-Chest/Working Paper - 2026 - Drechsler et al. - Credit Crunches and the Great Stagflation.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Working Paper - 2026 - Malenko et al. - Fragmentation of Shareholder Power</t>
+          <t>Working Paper - 2026 - Chen and Sacerdote - Capital in the Capitol Congressional Trades Resemble Uninformed Retail Trading</t>
         </is>
       </c>
       <c r="B4" s="2" t="n"/>
@@ -631,50 +631,50 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Malenko, Malenko, Tsoy</t>
+          <t>Chen, Sacerdote</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Fragmentation of Shareholder Power</t>
+          <t>Capital in the Capitol: Congressional Trades Resemble Uninformed Retail Trading</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>This paper develops a theoretical framework to evaluate how the asset-management industry's shift toward tailored portfolios, fund proliferation, and decentralized stewardship affects corporate governance. Growing heterogeneity in investor preferences better aligns products with demand but can fragment ownership and weaken managerial oversight. The authors show fund proliferation does not necessarily weaken governance: stronger manager incentives and concentrated portfolios of specialized funds can offset fragmentation, especially when investor preferences are intense. However, intense preferences can also push asset managers to compete by granting investors control—decentralizing stewardship and adopting pass-through voting—without internalizing the resulting governance costs. The paper clarifies when investor-driven customization helps or harms oversight.</t>
+          <t>This paper asks whether members of Congress exploit informational advantages in their personal stock trading, using a new hand-collected dataset of all U.S. legislators' and their families' trades from 2012 to 2023. After the STOCK Act, legislators' portfolios on average underperform or merely match market benchmarks. To explain this mediocre performance, the authors show legislators' positions track financial professionals' recommendations and that their trade timing reflects prevailing market sentiment - estimated from retail investors' social-media posts - rather than anticipating price moves. Congressional trading thus looks like public-signal-following and resembles uninformed retail behavior. The paper pushes back on the view that legislators systematically trade on private information.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>The paper begins from real industry trends—customization, more funds, and decentralized voting—and asks whether they necessarily erode the monitoring that concentrated ownership provides. It builds a model in which asset managers choose portfolio concentration, effort, and how much control to pass through to investors, given heterogeneous investor preferences. Analyzing the model, it shows proliferation can coexist with strong governance when incentives and specialization are strong, particularly under intense preferences. It then identifies a countervailing force: competition on the 'control' margin can lead managers to decentralize stewardship inefficiently, because they do not bear the full governance cost.</t>
+          <t>The paper revisits the contested question of congressional trading advantage, noting prior studies used limited samples and said little about mechanisms. It builds a comprehensive hand-collected record of legislator and family trades and evaluates performance against multiple benchmarks, finding no outperformance after the STOCK Act. It then probes why, testing whether trades follow analyst recommendations and align with market sentiment measured from retail social-media activity. Finding that timing mirrors public sentiment rather than leading prices, it concludes legislators' observable trading resembles uninformed retail trading.</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Theoretical model (mechanism/contracting framework) of asset-manager portfolio choice, incentives, and stewardship decentralization under heterogeneous investor preferences; no external dataset.</t>
+          <t>Event-study and calendar-time portfolio performance analysis on a hand-collected congressional-trading dataset, plus mechanism tests linking trades to analyst recommendations and social-media sentiment.</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>Corporate Governance, Asset Management, Financial Theory</t>
-        </is>
-      </c>
-      <c r="J4" s="2" t="inlineStr"/>
-      <c r="K4" s="2" t="inlineStr">
-        <is>
-          <t>Theoretical paper; no nonstandard datasets identified.</t>
-        </is>
-      </c>
+          <t>Political Economy, Informed Trading, Behavioral Finance</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Chen &amp; Sacerdote (this paper) — Congressional trading records; Context Analytics — S-Score (Twitter/X sentiment)</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="n"/>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>/home/runner/work/Knowledge-Chest/Knowledge-Chest/Working Paper - 2026 - Malenko et al. - Fragmentation of Shareholder Power.pdf</t>
+          <t>/home/runner/work/Knowledge-Chest/Knowledge-Chest/Working Paper - 2026 - Chen and Sacerdote - Capital in the Capitol Congressional Trades Resemble Uninformed Retail Trading.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Working Paper - 2026 - Bardóczy et al. - Monopsony Power and the Transmission of Monetary Policy</t>
+          <t>Working Paper - 2026 - Pagel et al. - Bank Fees and Household Financial Well-Being</t>
         </is>
       </c>
       <c r="B5" s="2" t="n"/>
@@ -683,50 +683,50 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Bardóczy, Bornstein, Salgado</t>
+          <t>Pagel, Sridhar, Williams</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Monopsony Power and the Transmission of Monetary Policy</t>
+          <t>Bank Fees and Household Financial Well-Being</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>This paper studies how employer labor-market power changes the way monetary policy transmits to wages and employment. Using administrative U.S. Census data, the authors show that high-monopsony firms—those accounting for over 10 percent of their local wage bill—adjust their wage bill and employment less in response to monetary policy. They rationalize this with a New Keynesian model featuring heterogeneous firms and oligopsonistic labor competition, where wage stickiness combined with labor-market power drives the muted response. The model isolates two channels—partial passthrough and misallocation—through which oligopsony shapes aggregate effects. Calibrated to U.S. labor markets, it implies that the decline in labor-market power since the 1980s raised the output response to monetary policy by about 10 percent and accounts for roughly 15 percent of the flattening of the Phillips curve.</t>
+          <t>This paper studies 2017-2022 policy changes at large U.S. banks that eliminated non-sufficient-funds (NSF) fees and relaxed overdraft policies, using individual transaction-level data. Eliminating NSF fees immediately reduced NSF charges across the income distribution, as expected. Relaxing overdraft policies, however, reduced overdraft fees only for wealthier (higher-income, higher-liquidity) households, and only they saw subsequent declines in late fees, interest, maintenance fees, and use of alternatives like payday loans. The authors conclude the changes were not substantial enough to meaningfully relieve financial stress for the most vulnerable households. Methodologically, the multi-treatment, varying-intensity setting motivates a new stacked event-study estimator related to de Chaisemartin et al. (2024) to handle staggered-DiD biases.</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>The paper posits that firms with labor-market power set wages strategically, so their response to monetary policy may differ systematically from competitive firms. Using administrative data, it establishes that high-monopsony firms adjust wage bill and employment less after monetary shocks. To interpret this, it builds a heterogeneous-firm New Keynesian model with oligopsony in which wage stickiness and market power jointly generate the muted response. The model formalizes partial passthrough and misallocation channels, and its calibration links the secular decline in monopsony to changes in the potency of monetary policy and the slope of the Phillips curve.</t>
+          <t>The paper asks whether widely publicized reductions in bank fees actually improved household financial well-being, especially for vulnerable households. Using transaction-level data, it separates two distinct policy changes - NSF-fee elimination and overdraft relaxation - and traces their effects across the income and liquidity distribution. It finds broad relief from NSF elimination but overdraft benefits accruing only to wealthier households, who then experience knock-on reductions in other fees and costly credit. Because the setting has multiple staggered treatments of differing intensity, it develops and applies a stacked event-study estimator to obtain unbiased effects.</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Empirical estimation of firm-level monetary-policy responses by monopsony intensity using administrative Census data, combined with a calibrated heterogeneous-firm New Keynesian model with oligopsonistic labor markets.</t>
+          <t>Stacked event-study / staggered difference-in-differences (a new estimator related to de Chaisemartin et al. 2024) on individual transaction-level banking data around NSF/overdraft policy changes.</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>Monetary Policy, Labor Market Power, Macroeconomics</t>
+          <t>Household Finance, Banking, Consumer Protection</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>U.S. Census Bureau — LEHD merged with Longitudinal Business Database (LBD)</t>
+          <t>Consumer transaction-data provider; FDIC — Summary of Deposits</t>
         </is>
       </c>
       <c r="K5" s="2" t="n"/>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>/home/runner/work/Knowledge-Chest/Knowledge-Chest/Working Paper - 2026 - Bardóczy et al. - Monopsony Power and the Transmission of Monetary Policy.pdf</t>
+          <t>/home/runner/work/Knowledge-Chest/Knowledge-Chest/Working Paper - 2026 - Pagel et al. - Bank Fees and Household Financial Well-Being.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Working Paper - 2026 - Thesmar and Verner - Beliefs and Stock Market Fluctuations New Evidence from the Past Seven Decades</t>
+          <t>Working Paper - 2026 - Matvos et al. - Private Credit, Balance Sheets and Financial Stability</t>
         </is>
       </c>
       <c r="B6" s="2" t="n"/>
@@ -735,50 +735,50 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Thesmar, Verner</t>
+          <t>Matvos, Piskorski, Seru</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Beliefs and Stock Market Fluctuations: New Evidence from the Past Seven Decades</t>
+          <t>Private Credit, Balance Sheets and Financial Stability</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>This paper builds a new seven-decade series of subjective expected equity returns (1956-2024) from an independent equity-analysis firm and uses it to reassess how beliefs move markets. Unlike the expectations of individual investors and professional forecasters, this measure is strongly positively correlated with the earnings-price ratio, responds negatively to past returns, and positively predicts future returns. Individual and professional-forecaster expectations are only weakly or negatively correlated with the new series, and disagreement between sophisticated and individual investors is associated with higher trading volume. The evidence fits a model of heterogeneous beliefs in which naive investors extrapolate past returns while sophisticated investors are close to rational. The paper offers a rare long-run window on the belief dynamics behind valuations.</t>
+          <t>This paper uses new, comprehensive fund- and asset-level data covering most of the private-credit industry to assess its balance sheets and financial-stability implications. Private-credit funds are highly capitalized, with equity typically 65-80% of assets - more than six times the capitalization of U.S. banks - and use only moderate debt, largely bank credit lines for liquidity management. Fund lives of 10-12 years exceed the shorter maturities of underlying loans, implying little maturity mismatch, unlike banks that fund long-term assets with short-term callable deposits. Portfolios are diversified across industries, geographies, and strategies, and performance shows positive average net returns with losses borne mainly by equity. The authors conclude that, as currently structured, private-credit funds are conservatively built and unlikely to pose bank-like systemic risks.</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>The paper motivates the need for a long, consistent measure of sophisticated investors' return expectations, which it constructs by hand from decades of an independent equity-analysis firm's forecasts. It characterizes the new series' properties—co-movement with the earnings-price ratio, mean-reverting response to past returns, and predictive power for future returns—and contrasts them with survey measures of individuals and forecasters. Finding that sophisticated and naive expectations diverge, and that their disagreement tracks trading volume, it argues a single-belief model cannot fit the facts. It then shows a heterogeneous-beliefs model, with extrapolative naive investors and near-rational sophisticated investors, rationalizes the joint patterns.</t>
+          <t>The paper addresses the financial-stability debate around private credit by bringing comprehensive fund- and asset-level data to bear on how these funds are actually capitalized and funded. It documents high equity ratios and limited, liquidity-oriented debt, contrasting this with banks' thin capital and deposit funding. It then shows the maturity structure implies little mismatch and that portfolios are diversified, limiting correlated-shock exposure. Finally it examines performance and loss-bearing, arguing the equity-heavy structure absorbs losses, so current private-credit configurations are unlikely to generate bank-style systemic risk.</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Construction and analysis of a novel long-run (1956-2024) subjective-expected-return series hand-collected from an independent equity-analysis firm, with predictive and correlation regressions against survey expectations and a heterogeneous-beliefs asset-pricing model.</t>
+          <t>Descriptive analysis of new proprietary fund- and asset-level private-credit data (~1,300 funds), benchmarked against U.S. commercial banks using regulatory data.</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>Behavioral Finance, Asset Pricing, Expectations &amp; Beliefs</t>
+          <t>Private Credit, Financial Stability, Banking</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Value Line Investment Survey; Robert Shiller — Investor Confidence Survey; UBS/Gallup and Livingston Survey</t>
+          <t>Proprietary private-credit data provider; Preqin</t>
         </is>
       </c>
       <c r="K6" s="2" t="n"/>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>/home/runner/work/Knowledge-Chest/Knowledge-Chest/Working Paper - 2026 - Thesmar and Verner - Beliefs and Stock Market Fluctuations New Evidence from the Past Seven Decades.pdf</t>
+          <t>/home/runner/work/Knowledge-Chest/Knowledge-Chest/Working Paper - 2026 - Matvos et al. - Private Credit, Balance Sheets and Financial Stability.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Working Paper - 2026 - Ahern - Industrial Concentration, Property Values, and Municipal Bond Spreads</t>
+          <t>Working Paper - 2026 - Baslandze et al. - Artificial Intelligence, Productivity, and the Workforce Evidence from Corporate Executives</t>
         </is>
       </c>
       <c r="B7" s="2" t="n"/>
@@ -787,50 +787,50 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Ahern</t>
+          <t>Baslandze, Edwards, Graham, McClure, Meyer, Sparks, Waddell, Weitz</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Industrial Concentration, Property Values, and Municipal Bond Spreads</t>
+          <t>Artificial Intelligence, Productivity, and the Workforce: Evidence from Corporate Executives</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>This paper shows that the industrial composition of a city's economy shapes its cost of municipal borrowing. In a panel of 1,177 U.S. cities from 2005 to 2022, greater sectoral concentration raises default risk and municipal bond spreads, especially where dominant industries are associated with low property values. Instrumental variables built from national sector-employment trends and regional house-price variation support a causal reading. A calibrated city-default model implies the estimated spread effect understates the gross risk from concentration, because concentration also brings agglomeration benefits that lower spreads, particularly in high-property-value cities. The paper connects local economic structure to public finance and credit risk.</t>
+          <t>This paper uses a novel survey of nearly 750 corporate executives to study how artificial intelligence is affecting productivity and the workforce. Adoption is highly heterogeneous: more than half of firms have already invested, though many smaller firms are just starting. Labor-productivity gains are positive, vary by sector, are expected to strengthen in 2026, and are concentrated in high-skill services and finance; they reflect higher revenue-based total factor productivity through innovation and demand channels rather than capital deepening. The authors document a 'productivity paradox' in which perceived gains exceed measured gains, likely due to delayed revenue realization. In labor markets they find little near-term aggregate employment decline, though large firms anticipate AI-driven reductions while smaller firms expect modest gains, alongside compositional labor reallocation.</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>The paper reasons that a city dependent on few industries faces more concentrated economic risk, which should raise default probability and hence bond spreads, but that the effect may depend on whether those industries support high property values that anchor the tax base. It documents the concentration–spread relationship in a large city panel and shows it is stronger where dominant sectors imply low property values. To move from correlation to causation, it instruments concentration using national sector-employment trends interacted with regional house-price variation. Finally, a calibrated default model reconciles the estimates with offsetting agglomeration benefits, implying the gross risk effect is larger than the net spread effect suggests.</t>
+          <t>Because firm-level effects of AI are hard to observe in standard data, the paper gathers direct evidence by surveying corporate executives about adoption, productivity, and workforce plans. It first documents wide heterogeneity in adoption and then characterizes the size, sectoral pattern, and channels of productivity gains, attributing them to revenue-based TFP rather than capital deepening. It reconciles optimistic perceptions with smaller measured effects through a productivity paradox driven by lagged revenue. Finally it turns to labor, showing limited aggregate employment effects so far but divergent expectations and reallocation across firm size and worker types.</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Panel regressions with an instrumental-variables strategy (national sector-employment trends and regional house-price variation) linking industrial concentration to municipal bond spreads, complemented by a calibrated structural model of city default.</t>
+          <t>Survey-based descriptive and cross-sectional analysis of ~750 corporate executives, with comparisons of adoption, productivity, and workforce outcomes across firm size and sector.</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>Municipal Finance, Credit Risk, Urban &amp; Regional Economics</t>
+          <t>Economics of AI, Productivity, Labor Economics</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>MSRB — Municipal Securities Rulemaking Board trade data; U.S. Census Bureau — LODES (LEHD Origin-Destination Employment Statistics); FHFA — House Price Index</t>
+          <t>Federal Reserve Bank of Atlanta &amp; Duke University — Survey of corporate executives</t>
         </is>
       </c>
       <c r="K7" s="2" t="n"/>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>/home/runner/work/Knowledge-Chest/Knowledge-Chest/Working Paper - 2026 - Ahern - Industrial Concentration, Property Values, and Municipal Bond Spreads.pdf</t>
+          <t>/home/runner/work/Knowledge-Chest/Knowledge-Chest/Working Paper - 2026 - Baslandze et al. - Artificial Intelligence, Productivity, and the Workforce Evidence from Corporate Executives.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Working Paper - 2026 - Clayton and Coppola - The Optimal Use of AI in Financial Regulation</t>
+          <t>Working Paper - 2026 - Eisfeldt et al. - Intangible Intensity</t>
         </is>
       </c>
       <c r="B8" s="2" t="n"/>
@@ -839,50 +839,50 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Clayton, Coppola</t>
+          <t>Eisfeldt, Hartman-Glaser, Kim, Lee</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>The Optimal Use of AI in Financial Regulation</t>
+          <t>Intangible Intensity</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>This paper asks whether modern AI methods applied to granular portfolio-holdings data can improve macroprudential regulation, and how policymakers should use such tools. The authors build a graph-based deep learning model over security-level holdings of financial intermediaries that embeds economic priors and learns latent representations of both assets and investors from the network of positions. Applied to the near-universe of non-bank financial intermediaries (about $40 trillion), the model forecasts intermediary trading far better than existing approaches, including during crises, and has more than ten times the explanatory power for cross-sectional stress-period returns. Its learned embeddings encode economically interpretable information about fire-sale vulnerability, and the architecture is inductive enough to produce estimates even for withheld asset classes or investors. The authors then embed the empirical model in a macroprudential optimal-policy framework, addressing the Lucas critique, to show why these objects matter for welfare.</t>
+          <t>This paper builds a text-based measure of firms' intangible investment intensity from 10-K filings and introduces a general 'semantic theme scoring' (STS) methodology. The approach further decomposes disclosure text into knowledge, customer, and organization capital. High-intangible-intensity firms are smaller, younger, and invest heavily in R&amp;D and human capital, and the three subcomponents map to distinct firm types - knowledge-intensive (R&amp;D-driven, high valuation, skilled labor), customer-intensive (mature, profitable, commercial), and organization-intensive (large, asset-heavy incumbents). The authors show managerial expenditure descriptions carry informative signals about intangible capital that complement financial statements. The paper offers both a new measure and a reusable NLP methodology for capturing corporate intangibles.</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>The paper frames systemic risk measurement as a prediction problem over the network of who holds what, arguing that the structure of intermediary holdings encodes fire-sale vulnerability that standard metrics miss. It develops a graph neural network with built-in economic priors that learns asset and investor representations from holdings, then validates the model out-of-sample on trading behavior and stress-period returns against existing benchmarks. Having shown the learned objects are predictive and interpretable, it asks how a regulator should optimally use them. It closes by embedding the empirical model in an equilibrium optimal-policy framework that confronts the Lucas critique, formalizing the welfare rationale for AI-based supervision.</t>
+          <t>The paper motivates that intangible capital is poorly captured by accounting statements, so it turns to the language firms use to describe their spending. It develops semantic theme scoring to convert 10-K disclosure text into an intangible-intensity measure and to separate knowledge, customer, and organization capital. It validates the measure by showing high-intangible firms have the expected profile and that the three components correspond to economically distinct firm types. It argues these text-derived signals complement financial data, opening avenues for measuring firms' position in the intangible lifecycle.</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Design and out-of-sample evaluation of a graph-based (network) deep-learning model on security-level intermediary holdings, benchmarked against existing systemic-risk metrics, embedded within a macroprudential optimal-policy framework robust to the Lucas critique.</t>
+          <t>Text-as-data measurement: a semantic-theme-scoring (NLP) methodology applied to 10-K filings to construct and validate an intangible-intensity measure and its subcomponents, with cross-sectional characterization.</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning in Finance, Financial Regulation, Systemic Risk</t>
+          <t>Intangible Capital, Text-as-Data / NLP, Corporate Finance</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>FactSet &amp; Morningstar — Security-level intermediary holdings</t>
+          <t>SEC (WRDS SEC Analytics Suite) — 10-K filings; S&amp;P Capital IQ</t>
         </is>
       </c>
       <c r="K8" s="2" t="n"/>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>/home/runner/work/Knowledge-Chest/Knowledge-Chest/Working Paper - 2026 - Clayton and Coppola - The Optimal Use of AI in Financial Regulation.pdf</t>
+          <t>/home/runner/work/Knowledge-Chest/Knowledge-Chest/Working Paper - 2026 - Eisfeldt et al. - Intangible Intensity.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Working Paper - 2026 - Ebsim et al. - Sophisticated Borrowing Constraints and Macroeconomic Dynamics</t>
+          <t>Working Paper - 2026 - Amiti et al. - Why Do Firms Pay Different Interest Rates on Their Bank Loans</t>
         </is>
       </c>
       <c r="B9" s="2" t="n"/>
@@ -891,50 +891,50 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Ebsim, Lian, Ma, Ottonello, Perez</t>
+          <t>Amiti, Kashyap, Kovner, Weinstein</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Sophisticated Borrowing Constraints and Macroeconomic Dynamics</t>
+          <t>Why Do Firms Pay Different Interest Rates on Their Bank Loans?</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>This paper argues that the way debt constraints are modeled fundamentally changes their macroeconomic implications. Traditional models impose hard borrowing limits that force firms to cut borrowing and investment whenever adverse shocks bind, producing financial acceleration. The authors instead model 'sophisticated borrowing constraints' resembling real-world financial covenants, where breaching an earnings-based debt threshold transfers control rights to creditors who then act to maximize their own value rather than mechanically shrinking credit. Calibrated to micro evidence on investment and earnings around covenant violations, the model matches firm-level dynamics while, at the macro level, generating no financial acceleration because violations do not trigger indiscriminate downscaling. The result challenges a workhorse mechanism linking credit conditions to aggregate fluctuations.</t>
+          <t>This paper documents large dispersion in interest rates on similar commercial and industrial loans using confidential supervisory data on the largest U.S. banks, and argues the spread is not explained by risk. The authors rationalize the dispersion with a search-cost model in which borrowers pay to solicit competing quotes. Estimated search costs are highest for smaller and riskier borrowers and lowest for public firms, matching predictable differences in screening and monitoring costs. The search costs are economically large: over a third of firms behave as if they never comparison-shop, half appear to obtain only two quotes, and the rest search widely. The paper interprets loan-rate dispersion as evidence of substantial search frictions in credit markets rather than pure risk pricing.</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>The paper contrasts textbook hard constraints, under which binding limits mechanically force deleveraging and amplify shocks, with the institutional reality of covenants, which reallocate control rather than dictate fixed borrowing ratios. It models covenant violation as a state-contingent transfer of control to creditors who choose firm policies to maximize creditor value, so tightening need not cause uniform credit cuts. The authors first show the model reproduces the empirical behavior of investment and earnings around violations at the micro level. They then embed the mechanism in a general-equilibrium setting and demonstrate that, unlike hard constraints, sophisticated constraints do not generate financial acceleration.</t>
+          <t>The paper starts from the puzzle that observably similar borrowers pay very different loan rates even after accounting for risk, suggesting frictions beyond credit quality. It proposes a search-cost model in which firms trade off the cost of gathering additional quotes against the rate savings, generating dispersion that depends on borrower type. Using confidential loan-level supervisory data, it strips out risk and attributes residual dispersion to search costs, which it estimates structurally. The estimated pattern - higher search costs for small, risky, private borrowers - lines up with the economics of screening and monitoring, and implies many firms effectively fail to shop around.</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>A quantitative macro-finance model with state-contingent, covenant-like borrowing constraints and creditor control rights, calibrated to firm-level dynamics around covenant violations, then evaluated for its aggregate (financial-acceleration) implications.</t>
+          <t>Structural estimation of a borrower search-cost model on confidential loan-level supervisory (FR Y-14) data, after controlling for risk, to recover the distribution of search costs across borrower types.</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>Macro-Finance, Corporate Debt &amp; Covenants, Firm Investment</t>
+          <t>Banking, Credit Markets, Search Frictions</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Refinitiv LPC — DealScan; Greg Nini (Nini, Smith &amp; Sufi) — Financial covenant violation data</t>
+          <t>Federal Reserve — FR Y-14 supervisory data</t>
         </is>
       </c>
       <c r="K9" s="2" t="n"/>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>/home/runner/work/Knowledge-Chest/Knowledge-Chest/Working Paper - 2026 - Ebsim et al. - Sophisticated Borrowing Constraints and Macroeconomic Dynamics.pdf</t>
+          <t>/home/runner/work/Knowledge-Chest/Knowledge-Chest/Working Paper - 2026 - Amiti et al. - Why Do Firms Pay Different Interest Rates on Their Bank Loans.pdf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Working Paper - 2026 - Dou et al. - The Cost of Intermediary Market Power for Distressed Borrowers</t>
+          <t>Working Paper - 2026 - Dyck et al. - Venture Fraud</t>
         </is>
       </c>
       <c r="B10" s="2" t="n"/>
@@ -943,50 +943,50 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Dou, Wang, Wang</t>
+          <t>Dyck, Fang, Hebert, Xu</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>The Cost of Intermediary Market Power for Distressed Borrowers</t>
+          <t>Venture Fraud</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>This paper measures how much lender market power raises borrowing costs for firms in financial distress, who must raise urgent financing in thin, concentrated credit markets. The authors show that distressed borrowers pay very high loan spreads even after stripping out compensation for credit risk, liquidity risk, and ordinary loan-making costs. To decompose the residual, they build and estimate a dynamic game-theoretic model of distressed lending featuring latent demand heterogeneity, endogenous lender participation, creditor blocking power, and tacit collusion sustained by repeated syndication. Lender market power explains 533 basis points of risk-adjusted spreads in debtor-in-possession (DIP) loans and 300 basis points in highly speculative loans, with roughly 140 basis points from tacit collusion in each. Because this markup reduces survival-critical liquidity by 16–20%, market power emerges as a major, previously underappreciated source of financial-distress costs.</t>
+          <t>This paper assembles the first comprehensive sample of venture fraud - 614 U.S. venture-capital-backed startups founded since 2000 that faced fraud allegations - and studies its governance roots. Within a high-detection subsample of newly public firms, VC-backed firms are 54% more likely to face fraud charges than comparable non-VC-backed firms. Fraud is more likely where founders hold stronger control rights, more convex cash-flow rights, more investors, and more non-traditional investors, with founder-controlled boards 88% more likely to commit fraud than VC- or shared-control boards. Governance features predict fraud far better than founder characteristics, and hot funding conditions at the first round - which weaken governance - forecast later fraud. The paper reframes venture fraud as substantially a product of governance structures rather than individual bad actors.</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>The argument begins by noting that distressed firms borrow in markets dominated by a few specialized lenders and by existing creditors who hold blocking power, so observed spreads may reflect market power rather than pure risk. The authors first document that DIP and highly speculative loan spreads remain large after removing risk and cost components, motivating a structural explanation. They then specify a dynamic game in which lenders choose whether to participate, exploit blocking power, and sustain tacit collusion through repeated syndication, allowing the markup to be identified and decomposed. Estimating the model on facility-level loan data, they quantify the market-power markup and trace its consequences for borrower liquidity and asset-value destruction.</t>
+          <t>The paper begins by building a large hand-collected sample of venture-fraud cases, addressing the measurement gap that has limited prior work. It first establishes that VC backing is associated with more fraud in a setting where detection is high and roughly uniform, ruling out pure detection differences. It then turns to mechanisms, arguing that founder-friendly structures and cap-table complexity weaken the monitoring that should deter fraud. Using a panel prediction model, it shows governance variables - founder control, convex payoffs, investor composition - dominate founder traits, and that hot-market financing conditions that erode governance at inception predict future fraud.</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Structural estimation of a dynamic game-theoretic model of distressed lending (with endogenous participation, creditor blocking power, and tacit collusion), disciplined by facility-level DIP and highly speculative loan data, used to decompose risk-adjusted spreads into market-power components.</t>
+          <t>Hand-collected case-sample construction plus a matched comparison (VC vs. non-VC among newly public firms) and a hazard-style panel prediction model relating fraud to governance and financing-market conditions.</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>Financial Distress &amp; Bankruptcy, Banking &amp; Lending, Market Power / Industrial Organization</t>
+          <t>Venture Capital, Corporate Governance, Financial Fraud</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>Refinitiv LPC — DealScan; LPC (Refinitiv) — LSTA/LPC Mark-to-Market Pricing Data; PACER — Public Access to Court Electronic Records; Moody's — Default and Recovery Database</t>
+          <t>PitchBook; Crunchbase; Dyck, Fang, Hebert &amp; Xu (this paper) — Venture-fraud case sample</t>
         </is>
       </c>
       <c r="K10" s="2" t="n"/>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>/home/runner/work/Knowledge-Chest/Knowledge-Chest/Working Paper - 2026 - Dou et al. - The Cost of Intermediary Market Power for Distressed Borrowers.pdf</t>
+          <t>/home/runner/work/Knowledge-Chest/Knowledge-Chest/Working Paper - 2026 - Dyck et al. - Venture Fraud.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Working Paper - 2026 - He et al. - Homemade Foreign Trading</t>
+          <t>Working Paper - 2026 - Diwan et al. - Competition and Fraud in Health Care</t>
         </is>
       </c>
       <c r="B11" s="2" t="n"/>
@@ -995,48 +995,568 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>He, Wang, Zhu</t>
+          <t>Diwan, Eliason, League, Leder-Luis, McDevitt, Roberts</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Homemade Foreign Trading</t>
+          <t>Competition and Fraud in Health Care</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>This paper documents how Chinese mainland insiders disguise domestic trades as foreign investment by round-tripping capital through the Stock Connect program, a practice the authors term 'homemade foreign trading.' Using cross-border holding data from all custodians in Stock Connect, they show that northbound flows predict returns and correlate with insider trading, but that this predictability decays after the 2018 Northbound Investor Identification reform introduced see-through surveillance. The decay is concentrated among less prestigious foreign custodians and cross-operating mainland custodians, precisely where insiders can most easily hide. The reform also reduces price informativeness in stocks most exposed to homemade foreign investors. The paper highlights regulatory cooperation as a key ingredient for the integrity of cross-border capital market integration.</t>
+          <t>This paper examines how competition affects fraud when governments procure goods and services from private firms, using Medicare's durable medical equipment (DME) market. The authors argue competition has an ambiguous effect on fraud: it dissipates the rents that attract fraudulent firms, but also squeezes margins so that legitimate firms may exit. Exploiting Medicare's switch from administratively regulated prices to competitive bidding for DME, they show that fraudulent suppliers' cost advantage let them gain market share while legitimate suppliers left the market. The result implies that price competition can perversely concentrate a market in fraudulent providers. The paper connects procurement design to the composition of firms and the prevalence of fraud.</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>The paper starts from the observation that Stock Connect lets mainland capital exit and re-enter disguised as foreign 'northbound' flow, giving insiders a channel to trade on private information while appearing to be offshore investors. It argues that if such round-tripping is real, northbound flows should predict returns and track insider activity, and that a reform imposing investor-level identification should break this link by making insiders identifiable. Exploiting the 2018 Northbound Investor Identification reform as a shock to surveillance, the authors trace how return predictability and its correlation with insider trading decay afterward. They then sharpen identification by showing the effect is strongest where hiding is easiest (opaque custodians) and by documenting a decline in price informativeness for the most exposed stocks.</t>
+          <t>The paper frames government procurement as a setting where competition lowers prices but may change which firms survive, since fraudulent firms have an artificial cost advantage from not delivering legitimate goods or services. It uses Medicare's DME competitive-bidding reform as a shock that sharply lowered reimbursement, predicting that legitimate suppliers with real costs are squeezed out while fraudulent suppliers persist. Linking supplier-level Medicare claims to fraud-enforcement records, it traces how market shares and exit differ between fraudulent and legitimate firms after the reform. It interprets the resulting shift as evidence that competition alone does not discipline fraud and can even entrench it.</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Event-study / difference-in-differences around the 2018 Northbound Investor Identification reform, using custodian-level cross-border holding data and return-predictability regressions, with cross-sectional heterogeneity by custodian type and stock exposure for identification.</t>
+          <t>Event-study/difference-in-differences around Medicare's switch to competitive bidding for durable medical equipment, using supplier-level claims linked to fraud-enforcement outcomes to compare fraudulent and legitimate firms.</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>International Finance, Insider Trading, Market Microstructure</t>
+          <t>Health Economics, Industrial Organization &amp; Procurement, Fraud &amp; Enforcement</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>China Securities Depository and Clearing (CSDC) / Stock Connect; CSMAR — China Stock Market &amp; Accounting Research; WIND</t>
+          <t>Centers for Medicare &amp; Medicaid Services (CMS) — Medicare DMEPOS claims; DOJ / HHS-OIG — Fraud enforcement records; Yunan Ji — Medicare DME auction bids</t>
         </is>
       </c>
       <c r="K11" s="2" t="n"/>
       <c r="L11" s="2" t="inlineStr">
         <is>
+          <t>/home/runner/work/Knowledge-Chest/Knowledge-Chest/Working Paper - 2026 - Diwan et al. - Competition and Fraud in Health Care.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Working Paper - 2026 - Correia et al. - Bank Runs with and without Bank Failure</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n"/>
+      <c r="C12" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Correia, Luck, Verner</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Bank Runs with and without Bank Failure</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>This paper builds a comprehensive historical database of U.S. bank runs by applying large language models to historical newspapers, yielding information on 3,984 runs on individual banks from 1863 to 1934. The data show runs are far more likely at weak banks but also occur at strong banks, especially following negative news about the real economy or the broader banking system. Crucially, runs typically cause failure only when a bank's fundamentals are poor; strong banks survive through signaling, interbank cooperation, and temporary suspension. Locally, runs on weak banks produce much larger declines in deposits, lending, and manufacturing activity than runs on strong banks. The findings put poor fundamentals at the center of both when runs occur and when they are economically damaging, tempering pure self-fulfilling-panic accounts.</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>The paper's first contribution is measurement: it uses LLMs to read historical newspapers and assemble a large, bank-level database of runs spanning 1863-1934. With this data, it asks whether runs strike indiscriminately or track fundamentals, showing runs concentrate in weak banks yet can hit strong banks after adverse news. It then distinguishes runs from failures, documenting that strong banks survive runs via signaling, cooperation, and suspension, so that failure requires poor fundamentals. Finally it links runs to local real outcomes, showing damage is concentrated where fundamentals are weak, which it interprets as evidence against models where small shocks trigger discontinuous jumps to bad equilibria.</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Construction of a novel bank-level historical dataset via large language models applied to newspaper archives, combined with empirical analysis relating runs to bank fundamentals, survival mechanisms, and local real-economy outcomes.</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>Banking History, Financial Crises, Text-as-Data / LLMs</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Correia, Luck &amp; Verner (this paper) — Historical bank-run database; Library of Congress — Chronicling America; OCC — National bank call reports (Annual Report to Congress)</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="n"/>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>/home/runner/work/Knowledge-Chest/Knowledge-Chest/Working Paper - 2026 - Correia et al. - Bank Runs with and without Bank Failure.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Working Paper - 2026 - Bornstein and Castillo-Martinez - Firm Exit and Financial Frictions</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="n"/>
+      <c r="C13" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Bornstein, Castillo-Martinez</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Firm Exit and Financial Frictions</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>This paper examines whether financial frictions cause too many firms to fail, motivating government interventions that prevent closures during crises. The authors build a firm-dynamics model with incomplete financial markets and show that frictions generate excessive firm exit, with a key sufficient statistic being the marginal propensity to exit with debt. Using confidential U.S. Census data, they estimate the debt–exit relationship and use it to discipline the model. The calibrated model implies that eliminating financial frictions would cut firm exit from 9.3% to 5.0% and deliver welfare gains of 3.6% in consumption-equivalent terms, with costs that spike during financial crises but not during ordinary productivity recessions. Comparing government-guaranteed loans and grants, the paper quantifies the trade-off between fiscal cost and effectiveness in preventing excessive exit.</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>The paper starts from the policy fear that viable-but-constrained firms fail in crises, and asks when firm exit is actually inefficient. It develops a firm-dynamics model with incomplete markets in which financial frictions distort the exit margin, isolating the marginal propensity to exit with debt as the statistic governing dynamic inefficiency. It then estimates the debt–exit relationship in confidential Census data to discipline that statistic and calibrate the model. Using the calibrated model, it quantifies the welfare cost of frictions across crisis and non-crisis states and evaluates guaranteed loans versus grants as interventions.</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>A quantitative firm-dynamics model with incomplete financial markets, disciplined by a reduced-form debt–exit relationship estimated on confidential U.S. Census microdata, used for welfare analysis and policy (loan-guarantee vs. grant) comparison.</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>Firm Dynamics, Financial Frictions, Macroeconomic Policy</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>U.S. Census Bureau — Longitudinal Business Database (LBD); Bureau van Dijk — Orbis (Italy)</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="n"/>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>/home/runner/work/Knowledge-Chest/Knowledge-Chest/Working Paper - 2026 - Bornstein and Castillo-Martinez - Firm Exit and Financial Frictions.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Working Paper - 2026 - Malenko et al. - Fragmentation of Shareholder Power</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n"/>
+      <c r="C14" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Malenko, Malenko, Tsoy</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Fragmentation of Shareholder Power</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>This paper develops a theoretical framework to evaluate how the asset-management industry's shift toward tailored portfolios, fund proliferation, and decentralized stewardship affects corporate governance. Growing heterogeneity in investor preferences better aligns products with demand but can fragment ownership and weaken managerial oversight. The authors show fund proliferation does not necessarily weaken governance: stronger manager incentives and concentrated portfolios of specialized funds can offset fragmentation, especially when investor preferences are intense. However, intense preferences can also push asset managers to compete by granting investors control—decentralizing stewardship and adopting pass-through voting—without internalizing the resulting governance costs. The paper clarifies when investor-driven customization helps or harms oversight.</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>The paper begins from real industry trends—customization, more funds, and decentralized voting—and asks whether they necessarily erode the monitoring that concentrated ownership provides. It builds a model in which asset managers choose portfolio concentration, effort, and how much control to pass through to investors, given heterogeneous investor preferences. Analyzing the model, it shows proliferation can coexist with strong governance when incentives and specialization are strong, particularly under intense preferences. It then identifies a countervailing force: competition on the 'control' margin can lead managers to decentralize stewardship inefficiently, because they do not bear the full governance cost.</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Theoretical model (mechanism/contracting framework) of asset-manager portfolio choice, incentives, and stewardship decentralization under heterogeneous investor preferences; no external dataset.</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>Corporate Governance, Asset Management, Financial Theory</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr"/>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>Theoretical paper; no nonstandard datasets identified.</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>/home/runner/work/Knowledge-Chest/Knowledge-Chest/Working Paper - 2026 - Malenko et al. - Fragmentation of Shareholder Power.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Working Paper - 2026 - Bardóczy et al. - Monopsony Power and the Transmission of Monetary Policy</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n"/>
+      <c r="C15" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Bardóczy, Bornstein, Salgado</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Monopsony Power and the Transmission of Monetary Policy</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>This paper studies how employer labor-market power changes the way monetary policy transmits to wages and employment. Using administrative U.S. Census data, the authors show that high-monopsony firms—those accounting for over 10 percent of their local wage bill—adjust their wage bill and employment less in response to monetary policy. They rationalize this with a New Keynesian model featuring heterogeneous firms and oligopsonistic labor competition, where wage stickiness combined with labor-market power drives the muted response. The model isolates two channels—partial passthrough and misallocation—through which oligopsony shapes aggregate effects. Calibrated to U.S. labor markets, it implies that the decline in labor-market power since the 1980s raised the output response to monetary policy by about 10 percent and accounts for roughly 15 percent of the flattening of the Phillips curve.</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>The paper posits that firms with labor-market power set wages strategically, so their response to monetary policy may differ systematically from competitive firms. Using administrative data, it establishes that high-monopsony firms adjust wage bill and employment less after monetary shocks. To interpret this, it builds a heterogeneous-firm New Keynesian model with oligopsony in which wage stickiness and market power jointly generate the muted response. The model formalizes partial passthrough and misallocation channels, and its calibration links the secular decline in monopsony to changes in the potency of monetary policy and the slope of the Phillips curve.</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>Empirical estimation of firm-level monetary-policy responses by monopsony intensity using administrative Census data, combined with a calibrated heterogeneous-firm New Keynesian model with oligopsonistic labor markets.</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>Monetary Policy, Labor Market Power, Macroeconomics</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>U.S. Census Bureau — LEHD merged with Longitudinal Business Database (LBD)</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="n"/>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>/home/runner/work/Knowledge-Chest/Knowledge-Chest/Working Paper - 2026 - Bardóczy et al. - Monopsony Power and the Transmission of Monetary Policy.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Working Paper - 2026 - Thesmar and Verner - Beliefs and Stock Market Fluctuations New Evidence from the Past Seven Decades</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="n"/>
+      <c r="C16" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Thesmar, Verner</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Beliefs and Stock Market Fluctuations: New Evidence from the Past Seven Decades</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>This paper builds a new seven-decade series of subjective expected equity returns (1956-2024) from an independent equity-analysis firm and uses it to reassess how beliefs move markets. Unlike the expectations of individual investors and professional forecasters, this measure is strongly positively correlated with the earnings-price ratio, responds negatively to past returns, and positively predicts future returns. Individual and professional-forecaster expectations are only weakly or negatively correlated with the new series, and disagreement between sophisticated and individual investors is associated with higher trading volume. The evidence fits a model of heterogeneous beliefs in which naive investors extrapolate past returns while sophisticated investors are close to rational. The paper offers a rare long-run window on the belief dynamics behind valuations.</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>The paper motivates the need for a long, consistent measure of sophisticated investors' return expectations, which it constructs by hand from decades of an independent equity-analysis firm's forecasts. It characterizes the new series' properties—co-movement with the earnings-price ratio, mean-reverting response to past returns, and predictive power for future returns—and contrasts them with survey measures of individuals and forecasters. Finding that sophisticated and naive expectations diverge, and that their disagreement tracks trading volume, it argues a single-belief model cannot fit the facts. It then shows a heterogeneous-beliefs model, with extrapolative naive investors and near-rational sophisticated investors, rationalizes the joint patterns.</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Construction and analysis of a novel long-run (1956-2024) subjective-expected-return series hand-collected from an independent equity-analysis firm, with predictive and correlation regressions against survey expectations and a heterogeneous-beliefs asset-pricing model.</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>Behavioral Finance, Asset Pricing, Expectations &amp; Beliefs</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>Value Line Investment Survey; Robert Shiller — Investor Confidence Survey; UBS/Gallup and Livingston Survey</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="n"/>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>/home/runner/work/Knowledge-Chest/Knowledge-Chest/Working Paper - 2026 - Thesmar and Verner - Beliefs and Stock Market Fluctuations New Evidence from the Past Seven Decades.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Working Paper - 2026 - Ahern - Industrial Concentration, Property Values, and Municipal Bond Spreads</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="n"/>
+      <c r="C17" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Ahern</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Industrial Concentration, Property Values, and Municipal Bond Spreads</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>This paper shows that the industrial composition of a city's economy shapes its cost of municipal borrowing. In a panel of 1,177 U.S. cities from 2005 to 2022, greater sectoral concentration raises default risk and municipal bond spreads, especially where dominant industries are associated with low property values. Instrumental variables built from national sector-employment trends and regional house-price variation support a causal reading. A calibrated city-default model implies the estimated spread effect understates the gross risk from concentration, because concentration also brings agglomeration benefits that lower spreads, particularly in high-property-value cities. The paper connects local economic structure to public finance and credit risk.</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>The paper reasons that a city dependent on few industries faces more concentrated economic risk, which should raise default probability and hence bond spreads, but that the effect may depend on whether those industries support high property values that anchor the tax base. It documents the concentration–spread relationship in a large city panel and shows it is stronger where dominant sectors imply low property values. To move from correlation to causation, it instruments concentration using national sector-employment trends interacted with regional house-price variation. Finally, a calibrated default model reconciles the estimates with offsetting agglomeration benefits, implying the gross risk effect is larger than the net spread effect suggests.</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>Panel regressions with an instrumental-variables strategy (national sector-employment trends and regional house-price variation) linking industrial concentration to municipal bond spreads, complemented by a calibrated structural model of city default.</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>Municipal Finance, Credit Risk, Urban &amp; Regional Economics</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>MSRB — Municipal Securities Rulemaking Board trade data; U.S. Census Bureau — LODES (LEHD Origin-Destination Employment Statistics); FHFA — House Price Index</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="n"/>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>/home/runner/work/Knowledge-Chest/Knowledge-Chest/Working Paper - 2026 - Ahern - Industrial Concentration, Property Values, and Municipal Bond Spreads.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Working Paper - 2026 - Clayton and Coppola - The Optimal Use of AI in Financial Regulation</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="n"/>
+      <c r="C18" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Clayton, Coppola</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>The Optimal Use of AI in Financial Regulation</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>This paper asks whether modern AI methods applied to granular portfolio-holdings data can improve macroprudential regulation, and how policymakers should use such tools. The authors build a graph-based deep learning model over security-level holdings of financial intermediaries that embeds economic priors and learns latent representations of both assets and investors from the network of positions. Applied to the near-universe of non-bank financial intermediaries (about $40 trillion), the model forecasts intermediary trading far better than existing approaches, including during crises, and has more than ten times the explanatory power for cross-sectional stress-period returns. Its learned embeddings encode economically interpretable information about fire-sale vulnerability, and the architecture is inductive enough to produce estimates even for withheld asset classes or investors. The authors then embed the empirical model in a macroprudential optimal-policy framework, addressing the Lucas critique, to show why these objects matter for welfare.</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>The paper frames systemic risk measurement as a prediction problem over the network of who holds what, arguing that the structure of intermediary holdings encodes fire-sale vulnerability that standard metrics miss. It develops a graph neural network with built-in economic priors that learns asset and investor representations from holdings, then validates the model out-of-sample on trading behavior and stress-period returns against existing benchmarks. Having shown the learned objects are predictive and interpretable, it asks how a regulator should optimally use them. It closes by embedding the empirical model in an equilibrium optimal-policy framework that confronts the Lucas critique, formalizing the welfare rationale for AI-based supervision.</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>Design and out-of-sample evaluation of a graph-based (network) deep-learning model on security-level intermediary holdings, benchmarked against existing systemic-risk metrics, embedded within a macroprudential optimal-policy framework robust to the Lucas critique.</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>Machine Learning in Finance, Financial Regulation, Systemic Risk</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>FactSet &amp; Morningstar — Security-level intermediary holdings</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="n"/>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>/home/runner/work/Knowledge-Chest/Knowledge-Chest/Working Paper - 2026 - Clayton and Coppola - The Optimal Use of AI in Financial Regulation.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Working Paper - 2026 - Ebsim et al. - Sophisticated Borrowing Constraints and Macroeconomic Dynamics</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="n"/>
+      <c r="C19" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Ebsim, Lian, Ma, Ottonello, Perez</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Sophisticated Borrowing Constraints and Macroeconomic Dynamics</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>This paper argues that the way debt constraints are modeled fundamentally changes their macroeconomic implications. Traditional models impose hard borrowing limits that force firms to cut borrowing and investment whenever adverse shocks bind, producing financial acceleration. The authors instead model 'sophisticated borrowing constraints' resembling real-world financial covenants, where breaching an earnings-based debt threshold transfers control rights to creditors who then act to maximize their own value rather than mechanically shrinking credit. Calibrated to micro evidence on investment and earnings around covenant violations, the model matches firm-level dynamics while, at the macro level, generating no financial acceleration because violations do not trigger indiscriminate downscaling. The result challenges a workhorse mechanism linking credit conditions to aggregate fluctuations.</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>The paper contrasts textbook hard constraints, under which binding limits mechanically force deleveraging and amplify shocks, with the institutional reality of covenants, which reallocate control rather than dictate fixed borrowing ratios. It models covenant violation as a state-contingent transfer of control to creditors who choose firm policies to maximize creditor value, so tightening need not cause uniform credit cuts. The authors first show the model reproduces the empirical behavior of investment and earnings around violations at the micro level. They then embed the mechanism in a general-equilibrium setting and demonstrate that, unlike hard constraints, sophisticated constraints do not generate financial acceleration.</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>A quantitative macro-finance model with state-contingent, covenant-like borrowing constraints and creditor control rights, calibrated to firm-level dynamics around covenant violations, then evaluated for its aggregate (financial-acceleration) implications.</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>Macro-Finance, Corporate Debt &amp; Covenants, Firm Investment</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>Refinitiv LPC — DealScan; Greg Nini (Nini, Smith &amp; Sufi) — Financial covenant violation data</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="n"/>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>/home/runner/work/Knowledge-Chest/Knowledge-Chest/Working Paper - 2026 - Ebsim et al. - Sophisticated Borrowing Constraints and Macroeconomic Dynamics.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Working Paper - 2026 - Dou et al. - The Cost of Intermediary Market Power for Distressed Borrowers</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="n"/>
+      <c r="C20" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Dou, Wang, Wang</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>The Cost of Intermediary Market Power for Distressed Borrowers</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>This paper measures how much lender market power raises borrowing costs for firms in financial distress, who must raise urgent financing in thin, concentrated credit markets. The authors show that distressed borrowers pay very high loan spreads even after stripping out compensation for credit risk, liquidity risk, and ordinary loan-making costs. To decompose the residual, they build and estimate a dynamic game-theoretic model of distressed lending featuring latent demand heterogeneity, endogenous lender participation, creditor blocking power, and tacit collusion sustained by repeated syndication. Lender market power explains 533 basis points of risk-adjusted spreads in debtor-in-possession (DIP) loans and 300 basis points in highly speculative loans, with roughly 140 basis points from tacit collusion in each. Because this markup reduces survival-critical liquidity by 16–20%, market power emerges as a major, previously underappreciated source of financial-distress costs.</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>The argument begins by noting that distressed firms borrow in markets dominated by a few specialized lenders and by existing creditors who hold blocking power, so observed spreads may reflect market power rather than pure risk. The authors first document that DIP and highly speculative loan spreads remain large after removing risk and cost components, motivating a structural explanation. They then specify a dynamic game in which lenders choose whether to participate, exploit blocking power, and sustain tacit collusion through repeated syndication, allowing the markup to be identified and decomposed. Estimating the model on facility-level loan data, they quantify the market-power markup and trace its consequences for borrower liquidity and asset-value destruction.</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>Structural estimation of a dynamic game-theoretic model of distressed lending (with endogenous participation, creditor blocking power, and tacit collusion), disciplined by facility-level DIP and highly speculative loan data, used to decompose risk-adjusted spreads into market-power components.</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>Financial Distress &amp; Bankruptcy, Banking &amp; Lending, Market Power / Industrial Organization</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>Refinitiv LPC — DealScan; LPC (Refinitiv) — LSTA/LPC Mark-to-Market Pricing Data; PACER — Public Access to Court Electronic Records; Moody's — Default and Recovery Database</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="n"/>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>/home/runner/work/Knowledge-Chest/Knowledge-Chest/Working Paper - 2026 - Dou et al. - The Cost of Intermediary Market Power for Distressed Borrowers.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Working Paper - 2026 - He et al. - Homemade Foreign Trading</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="n"/>
+      <c r="C21" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>He, Wang, Zhu</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Homemade Foreign Trading</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>This paper documents how Chinese mainland insiders disguise domestic trades as foreign investment by round-tripping capital through the Stock Connect program, a practice the authors term 'homemade foreign trading.' Using cross-border holding data from all custodians in Stock Connect, they show that northbound flows predict returns and correlate with insider trading, but that this predictability decays after the 2018 Northbound Investor Identification reform introduced see-through surveillance. The decay is concentrated among less prestigious foreign custodians and cross-operating mainland custodians, precisely where insiders can most easily hide. The reform also reduces price informativeness in stocks most exposed to homemade foreign investors. The paper highlights regulatory cooperation as a key ingredient for the integrity of cross-border capital market integration.</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>The paper starts from the observation that Stock Connect lets mainland capital exit and re-enter disguised as foreign 'northbound' flow, giving insiders a channel to trade on private information while appearing to be offshore investors. It argues that if such round-tripping is real, northbound flows should predict returns and track insider activity, and that a reform imposing investor-level identification should break this link by making insiders identifiable. Exploiting the 2018 Northbound Investor Identification reform as a shock to surveillance, the authors trace how return predictability and its correlation with insider trading decay afterward. They then sharpen identification by showing the effect is strongest where hiding is easiest (opaque custodians) and by documenting a decline in price informativeness for the most exposed stocks.</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>Event-study / difference-in-differences around the 2018 Northbound Investor Identification reform, using custodian-level cross-border holding data and return-predictability regressions, with cross-sectional heterogeneity by custodian type and stock exposure for identification.</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>International Finance, Insider Trading, Market Microstructure</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>China Securities Depository and Clearing (CSDC) / Stock Connect; CSMAR — China Stock Market &amp; Accounting Research; WIND</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="n"/>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
           <t>/home/runner/work/Knowledge-Chest/Knowledge-Chest/Working Paper - 2026 - He et al. - Homemade Foreign Trading.pdf</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L11"/>
+  <autoFilter ref="A1:L21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1047,7 +1567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1148,14 +1668,18 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>China Securities Depository and Clearing (CSDC) / Stock Connect</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr"/>
+          <t>Centers for Medicare &amp; Medicaid Services (CMS)</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Medicare DMEPOS claims</t>
+        </is>
+      </c>
       <c r="C3" s="2" t="inlineStr"/>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Cross-border holding and order data from all custodians in China's Stock Connect (northbound), including the 2018 Northbound Investor Identification reform, used to trace round-tripping insider flows.</t>
+          <t>Supplier- (NPI-) level Medicare durable medical equipment claims used to measure market shares, entry, and exit around the competitive-bidding reform.</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -1166,7 +1690,7 @@
       <c r="F3" s="2" t="inlineStr"/>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>China; Stock Connect; custodians; cross-border holdings</t>
+          <t>Medicare; DME; claims; suppliers</t>
         </is>
       </c>
       <c r="H3" s="2" t="n">
@@ -1174,25 +1698,25 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>Working Paper - 2026 - He et al. - Homemade Foreign Trading</t>
+          <t>Working Paper - 2026 - Diwan et al. - Competition and Fraud in Health Care</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Correia, Luck &amp; Verner (this paper)</t>
+          <t>Chen &amp; Sacerdote (this paper)</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Historical bank-run database</t>
+          <t>Congressional trading records</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr"/>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Newly constructed database of 3,984 bank runs on individual U.S. banks, 1863-1934, extracted from historical newspapers using large language models.</t>
+          <t>Hand-collected transactions of all U.S. members of Congress and their immediate families, 2012-2023, from periodic financial-disclosure (STOCK Act) filings.</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -1203,7 +1727,7 @@
       <c r="F4" s="2" t="inlineStr"/>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>bank runs; historical; LLM-constructed</t>
+          <t>congressional trades; disclosures; hand-collected</t>
         </is>
       </c>
       <c r="H4" s="2" t="n">
@@ -1211,36 +1735,32 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>Working Paper - 2026 - Correia et al. - Bank Runs with and without Bank Failure</t>
+          <t>Working Paper - 2026 - Chen and Sacerdote - Capital in the Capitol Congressional Trades Resemble Uninformed Retail Trading</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>CSMAR</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>China Stock Market &amp; Accounting Research</t>
-        </is>
-      </c>
+          <t>China Securities Depository and Clearing (CSDC) / Stock Connect</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr"/>
       <c r="C5" s="2" t="inlineStr"/>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Chinese firms' financial statements and corporate announcements used for firm characteristics and insider-trading events.</t>
+          <t>Cross-border holding and order data from all custodians in China's Stock Connect (northbound), including the 2018 Northbound Investor Identification reform, used to trace round-tripping insider flows.</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Proprietary</t>
+          <t>Restricted</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr"/>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>China; accounting; announcements</t>
+          <t>China; Stock Connect; custodians; cross-border holdings</t>
         </is>
       </c>
       <c r="H5" s="2" t="n">
@@ -1255,18 +1775,14 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>FactSet &amp; Morningstar</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Security-level intermediary holdings</t>
-        </is>
-      </c>
+          <t>Consumer transaction-data provider</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr"/>
       <c r="C6" s="2" t="inlineStr"/>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Holdings data covering the universe of non-bank financial intermediaries (mutual funds, ETFs, separate accounts, etc.), ~$40 trillion, used to train the holdings-network model.</t>
+          <t>Individual account- and transaction-level banking data used to measure NSF, overdraft, late, and maintenance fees and use of alternative financial services across households.</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -1277,7 +1793,7 @@
       <c r="F6" s="2" t="inlineStr"/>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>holdings network; non-bank intermediaries; fire sales</t>
+          <t>transaction-level; bank fees; households</t>
         </is>
       </c>
       <c r="H6" s="2" t="n">
@@ -1285,36 +1801,36 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>Working Paper - 2026 - Clayton and Coppola - The Optimal Use of AI in Financial Regulation</t>
+          <t>Working Paper - 2026 - Pagel et al. - Bank Fees and Household Financial Well-Being</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>FHFA</t>
+          <t>Context Analytics</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>House Price Index</t>
+          <t>S-Score (Twitter/X sentiment)</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr"/>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Regional house-price data (pre-sample 1975-2004) used to build instruments and proxy property values.</t>
+          <t>Security-level social-media sentiment scores derived from the Twitter/X firehose via proprietary NLP, used to proxy retail market sentiment.</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>Proprietary</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr"/>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>house prices; property values</t>
+          <t>social media sentiment; retail; NLP</t>
         </is>
       </c>
       <c r="H7" s="2" t="n">
@@ -1322,36 +1838,36 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>Working Paper - 2026 - Ahern - Industrial Concentration, Property Values, and Municipal Bond Spreads</t>
+          <t>Working Paper - 2026 - Chen and Sacerdote - Capital in the Capitol Congressional Trades Resemble Uninformed Retail Trading</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Greg Nini (Nini, Smith &amp; Sufi)</t>
+          <t>Correia, Luck &amp; Verner (this paper)</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Financial covenant violation data</t>
+          <t>Historical bank-run database</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr"/>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Hand-shared extended data on financial covenant violations disclosed in firms' filings, 1996 onward, used to construct micro moments around violations.</t>
+          <t>Newly constructed database of 3,984 bank runs on individual U.S. banks, 1863-1934, extracted from historical newspapers using large language models.</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Restricted</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr"/>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>covenant violations; control rights</t>
+          <t>bank runs; historical; LLM-constructed</t>
         </is>
       </c>
       <c r="H8" s="2" t="n">
@@ -1359,36 +1875,32 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>Working Paper - 2026 - Ebsim et al. - Sophisticated Borrowing Constraints and Macroeconomic Dynamics</t>
+          <t>Working Paper - 2026 - Correia et al. - Bank Runs with and without Bank Failure</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Library of Congress</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>Chronicling America</t>
-        </is>
-      </c>
+          <t>Crunchbase</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr"/>
       <c r="C9" s="2" t="inlineStr"/>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Large-scale archive of digitized historical U.S. newspapers, the main source for detecting and dating bank runs.</t>
+          <t>Startup and news-feed data used alongside PitchBook to identify fraud allegations.</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>Proprietary</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr"/>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>historical newspapers; text source</t>
+          <t>startups; news; allegations</t>
         </is>
       </c>
       <c r="H9" s="2" t="n">
@@ -1396,25 +1908,25 @@
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>Working Paper - 2026 - Correia et al. - Bank Runs with and without Bank Failure</t>
+          <t>Working Paper - 2026 - Dyck et al. - Venture Fraud</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>LPC (Refinitiv)</t>
+          <t>CSMAR</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>LSTA/LPC Mark-to-Market Pricing Data</t>
+          <t>China Stock Market &amp; Accounting Research</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr"/>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Secondary-market loan trading/pricing data used to measure loan liquidity and pricing.</t>
+          <t>Chinese firms' financial statements and corporate announcements used for firm characteristics and insider-trading events.</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -1425,7 +1937,7 @@
       <c r="F10" s="2" t="inlineStr"/>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>secondary loan prices; liquidity</t>
+          <t>China; accounting; announcements</t>
         </is>
       </c>
       <c r="H10" s="2" t="n">
@@ -1433,36 +1945,36 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>Working Paper - 2026 - Dou et al. - The Cost of Intermediary Market Power for Distressed Borrowers</t>
+          <t>Working Paper - 2026 - He et al. - Homemade Foreign Trading</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Moody's</t>
+          <t>DOJ / HHS-OIG</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Default and Recovery Database</t>
+          <t>Fraud enforcement records</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr"/>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Nominal recovery rates aggregated by industry, used in the risk-adjustment of spreads.</t>
+          <t>Federal fraud enforcement actions - indictments, civil settlements, and program exclusions - used to identify fraudulent suppliers.</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Proprietary</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr"/>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>defaults; recoveries</t>
+          <t>fraud enforcement; exclusions; indictments</t>
         </is>
       </c>
       <c r="H11" s="2" t="n">
@@ -1470,25 +1982,25 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>Working Paper - 2026 - Dou et al. - The Cost of Intermediary Market Power for Distressed Borrowers</t>
+          <t>Working Paper - 2026 - Diwan et al. - Competition and Fraud in Health Care</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>MSRB</t>
+          <t>Dyck, Fang, Hebert &amp; Xu (this paper)</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Municipal Securities Rulemaking Board trade data</t>
+          <t>Venture-fraud case sample</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr"/>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Secondary-market municipal bond trades used to construct city-level bond spreads.</t>
+          <t>Hand-collected sample of 614 U.S. VC-backed startups facing fraud charges (SEC, DOJ, and civil litigation) since 2000, with fraud commitment periods.</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -1499,7 +2011,7 @@
       <c r="F12" s="2" t="inlineStr"/>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>municipal bonds; spreads; secondary market</t>
+          <t>venture fraud; hand-collected; litigation</t>
         </is>
       </c>
       <c r="H12" s="2" t="n">
@@ -1507,36 +2019,36 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>Working Paper - 2026 - Ahern - Industrial Concentration, Property Values, and Municipal Bond Spreads</t>
+          <t>Working Paper - 2026 - Dyck et al. - Venture Fraud</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>OCC</t>
+          <t>FactSet &amp; Morningstar</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>National bank call reports (Annual Report to Congress)</t>
+          <t>Security-level intermediary holdings</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr"/>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Balance-sheet data for national banks used to measure bank fundamentals and outcomes.</t>
+          <t>Holdings data covering the universe of non-bank financial intermediaries (mutual funds, ETFs, separate accounts, etc.), ~$40 trillion, used to train the holdings-network model.</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>Proprietary</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr"/>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>call reports; bank balance sheets; fundamentals</t>
+          <t>holdings network; non-bank intermediaries; fire sales</t>
         </is>
       </c>
       <c r="H13" s="2" t="n">
@@ -1544,25 +2056,25 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>Working Paper - 2026 - Correia et al. - Bank Runs with and without Bank Failure</t>
+          <t>Working Paper - 2026 - Clayton and Coppola - The Optimal Use of AI in Financial Regulation</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>PACER</t>
+          <t>FDIC</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Public Access to Court Electronic Records</t>
+          <t>Summary of Deposits</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr"/>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>U.S. bankruptcy court records used to identify DIP financing and Chapter 11 cases.</t>
+          <t>Branch/deposit data used to determine which metropolitan areas were exposed to each bank's policy change.</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -1573,7 +2085,7 @@
       <c r="F14" s="2" t="inlineStr"/>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>bankruptcy; DIP; court records</t>
+          <t>deposits; branch exposure; MSA</t>
         </is>
       </c>
       <c r="H14" s="2" t="n">
@@ -1581,73 +2093,73 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>Working Paper - 2026 - Dou et al. - The Cost of Intermediary Market Power for Distressed Borrowers</t>
+          <t>Working Paper - 2026 - Pagel et al. - Bank Fees and Household Financial Well-Being</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Refinitiv LPC</t>
+          <t>FDIC</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>DealScan</t>
+          <t>Historical Bank Data</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr"/>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Loan-level covenant terms (e.g., debt-to-EBITDA covenants) used to identify firms subject to earnings-based constraints. Facility-level syndicated loan terms used to build the sample of debtor-in-possession and highly speculative loans.</t>
+          <t>Aggregate historical deposits and deposit interest expense used to characterize Reg Q-era bank funding.</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Proprietary</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr"/>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>syndicated loans; DIP; facilities; loan covenants; debt-to-EBITDA</t>
+          <t>historical deposits; Reg Q</t>
         </is>
       </c>
       <c r="H15" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>Working Paper - 2026 - Dou et al. - The Cost of Intermediary Market Power for Distressed Borrowers; Working Paper - 2026 - Ebsim et al. - Sophisticated Borrowing Constraints and Macroeconomic Dynamics</t>
+          <t>Working Paper - 2026 - Drechsler et al. - Credit Crunches and the Great Stagflation</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Robert Shiller</t>
+          <t>Federal Reserve</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Investor Confidence Survey</t>
+          <t>FR Y-14 supervisory data</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr"/>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Investor-confidence survey data used as a comparison measure of investor beliefs.</t>
+          <t>Confidential loan-level data on commercial and industrial loans at the largest U.S. banks, collected for Dodd-Frank stress testing, used to measure rate dispersion and borrower/loan characteristics.</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>Restricted</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr"/>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>investor confidence; beliefs</t>
+          <t>supervisory; C&amp;I loans; bank stress test</t>
         </is>
       </c>
       <c r="H16" s="2" t="n">
@@ -1655,25 +2167,25 @@
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>Working Paper - 2026 - Thesmar and Verner - Beliefs and Stock Market Fluctuations New Evidence from the Past Seven Decades</t>
+          <t>Working Paper - 2026 - Amiti et al. - Why Do Firms Pay Different Interest Rates on Their Bank Loans</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>U.S. Census Bureau</t>
+          <t>Federal Reserve</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>LODES (LEHD Origin-Destination Employment Statistics)</t>
+          <t>Senior Loan Officer Opinion Survey (SLOOS)</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr"/>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Sector-level job counts used to measure a city's industrial concentration.</t>
+          <t>Bank lending-standards survey (back to 1964) used as a measure of credit tightening.</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
@@ -1684,7 +2196,7 @@
       <c r="F17" s="2" t="inlineStr"/>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>employment; industry concentration; LODES</t>
+          <t>lending standards; SLOOS</t>
         </is>
       </c>
       <c r="H17" s="2" t="n">
@@ -1692,36 +2204,36 @@
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>Working Paper - 2026 - Ahern - Industrial Concentration, Property Values, and Municipal Bond Spreads</t>
+          <t>Working Paper - 2026 - Drechsler et al. - Credit Crunches and the Great Stagflation</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>U.S. Census Bureau</t>
+          <t>Federal Reserve Bank of Atlanta</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>LEHD merged with Longitudinal Business Database (LBD)</t>
+          <t>Diary of Consumer Payment Choice (DCPC)</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr"/>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Confidential administrative data on establishment-level wage bill and employment used to measure local monopsony power and firm responses to monetary policy.</t>
+          <t>Consumer payment-diary data on payment-method use and shopping, used to measure sorting across merchant sectors.</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Restricted</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr"/>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>administrative; wage bill; employment; monopsony</t>
+          <t>consumer payments; diary; sorting</t>
         </is>
       </c>
       <c r="H18" s="2" t="n">
@@ -1729,25 +2241,25 @@
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>Working Paper - 2026 - Bardóczy et al. - Monopsony Power and the Transmission of Monetary Policy</t>
+          <t>Working Paper - 2026 - Egan et al. - Who Pays for Payments</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>U.S. Census Bureau</t>
+          <t>Federal Reserve Bank of Atlanta &amp; Duke University</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Longitudinal Business Database (LBD)</t>
+          <t>Survey of corporate executives</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr"/>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Confidential data tracking entry and exit for the universe of U.S. employers, used to estimate the debt–exit relationship.</t>
+          <t>Novel survey of nearly 750 corporate executives on AI adoption, productivity effects, and workforce plans, benchmarked to the U.S. Census industry/size distribution.</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -1758,7 +2270,7 @@
       <c r="F19" s="2" t="inlineStr"/>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>firm entry/exit; universe of employers</t>
+          <t>executive survey; AI adoption; productivity</t>
         </is>
       </c>
       <c r="H19" s="2" t="n">
@@ -1766,21 +2278,25 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>Working Paper - 2026 - Bornstein and Castillo-Martinez - Firm Exit and Financial Frictions</t>
+          <t>Working Paper - 2026 - Baslandze et al. - Artificial Intelligence, Productivity, and the Workforce Evidence from Corporate Executives</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>UBS/Gallup and Livingston Survey</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr"/>
+          <t>FHFA</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>House Price Index</t>
+        </is>
+      </c>
       <c r="C20" s="2" t="inlineStr"/>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Survey measures of individual-investor and professional-forecaster return/earnings expectations used for comparison.</t>
+          <t>Regional house-price data (pre-sample 1975-2004) used to build instruments and proxy property values.</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -1791,7 +2307,7 @@
       <c r="F20" s="2" t="inlineStr"/>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>investor surveys; forecaster expectations</t>
+          <t>house prices; property values</t>
         </is>
       </c>
       <c r="H20" s="2" t="n">
@@ -1799,32 +2315,32 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>Working Paper - 2026 - Thesmar and Verner - Beliefs and Stock Market Fluctuations New Evidence from the Past Seven Decades</t>
+          <t>Working Paper - 2026 - Ahern - Industrial Concentration, Property Values, and Municipal Bond Spreads</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Value Line Investment Survey</t>
+          <t>Fiserv</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr"/>
       <c r="C21" s="2" t="inlineStr"/>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Analyst forecasts hand-collected from microfilm records (1956-2024) used to construct a long-run series of sophisticated investors' subjective expected returns.</t>
+          <t>Two proprietary datasets from Fiserv, a large U.S. merchant acquirer, on the composition and cost (interchange/settlement) of payments across merchants.</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Restricted</t>
+          <t>Proprietary</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr"/>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>subjective expectations; analyst forecasts; microfilm</t>
+          <t>merchant acquiring; interchange; settlement</t>
         </is>
       </c>
       <c r="H21" s="2" t="n">
@@ -1832,45 +2348,864 @@
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>Working Paper - 2026 - Thesmar and Verner - Beliefs and Stock Market Fluctuations New Evidence from the Past Seven Decades</t>
+          <t>Working Paper - 2026 - Egan et al. - Who Pays for Payments</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>WIND</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr"/>
+          <t>Greg Nini (Nini, Smith &amp; Sufi)</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Financial covenant violation data</t>
+        </is>
+      </c>
       <c r="C22" s="2" t="inlineStr"/>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Adjusted opening prices and free-floating shares for Chinese listed stocks.</t>
+          <t>Hand-shared extended data on financial covenant violations disclosed in firms' filings, 1996 onward, used to construct micro moments around violations.</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Proprietary</t>
+          <t>Restricted</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr"/>
       <c r="G22" s="2" t="inlineStr">
         <is>
+          <t>covenant violations; control rights</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>Working Paper - 2026 - Ebsim et al. - Sophisticated Borrowing Constraints and Macroeconomic Dynamics</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Library of Congress</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Chronicling America</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr"/>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Large-scale archive of digitized historical U.S. newspapers, the main source for detecting and dating bank runs.</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr"/>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>historical newspapers; text source</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>Working Paper - 2026 - Correia et al. - Bank Runs with and without Bank Failure</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>LPC (Refinitiv)</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>LSTA/LPC Mark-to-Market Pricing Data</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr"/>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Secondary-market loan trading/pricing data used to measure loan liquidity and pricing.</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Proprietary</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr"/>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>secondary loan prices; liquidity</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>Working Paper - 2026 - Dou et al. - The Cost of Intermediary Market Power for Distressed Borrowers</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Moody's</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Default and Recovery Database</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr"/>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Nominal recovery rates aggregated by industry, used in the risk-adjustment of spreads.</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>Proprietary</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr"/>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>defaults; recoveries</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>Working Paper - 2026 - Dou et al. - The Cost of Intermediary Market Power for Distressed Borrowers</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>MSRB</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Municipal Securities Rulemaking Board trade data</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr"/>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Secondary-market municipal bond trades used to construct city-level bond spreads.</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr"/>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>municipal bonds; spreads; secondary market</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>Working Paper - 2026 - Ahern - Industrial Concentration, Property Values, and Municipal Bond Spreads</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>NBER-CES</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Manufacturing Industry Database</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr"/>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Industry-level prices and quantities (derived from the U.S. Census) used to test cross-industry supply effects.</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr"/>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>manufacturing; prices; quantities</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>Working Paper - 2026 - Drechsler et al. - Credit Crunches and the Great Stagflation</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Nilson Report</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr"/>
+      <c r="C28" s="2" t="inlineStr"/>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Industry statistics on interchange and network fees used to benchmark payment costs.</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>Proprietary</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr"/>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>interchange; network fees; benchmarks</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>Working Paper - 2026 - Egan et al. - Who Pays for Payments</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>OCC</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>National bank call reports (Annual Report to Congress)</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr"/>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Balance-sheet data for national banks used to measure bank fundamentals and outcomes.</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr"/>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>call reports; bank balance sheets; fundamentals</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>Working Paper - 2026 - Correia et al. - Bank Runs with and without Bank Failure</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>PACER</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Public Access to Court Electronic Records</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr"/>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>U.S. bankruptcy court records used to identify DIP financing and Chapter 11 cases.</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr"/>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>bankruptcy; DIP; court records</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>Working Paper - 2026 - Dou et al. - The Cost of Intermediary Market Power for Distressed Borrowers</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>PitchBook</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr"/>
+      <c r="C31" s="2" t="inlineStr"/>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Venture-capital-backed startups, their founders, financing rounds, and cap-table/board structures, used to build the sample and governance variables.</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>Proprietary</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr"/>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>venture capital; startups; cap tables</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>Working Paper - 2026 - Dyck et al. - Venture Fraud</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Preqin</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr"/>
+      <c r="C32" s="2" t="inlineStr"/>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Industry-level private-credit assets used to gauge coverage and situate the sample within the broader market.</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Proprietary</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr"/>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>private credit; industry assets</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>Working Paper - 2026 - Matvos et al. - Private Credit, Balance Sheets and Financial Stability</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Proprietary private-credit data provider</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr"/>
+      <c r="C33" s="2" t="inlineStr"/>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>New proprietary fund- and asset-level data covering roughly 1,300 private-credit funds and their loans (capitalization, funding, maturities, performance), covering most of the industry.</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>Proprietary</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr"/>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>private credit; funds; balance sheets</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>Working Paper - 2026 - Matvos et al. - Private Credit, Balance Sheets and Financial Stability</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Refinitiv LPC</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>DealScan</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr"/>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Loan-level covenant terms (e.g., debt-to-EBITDA covenants) used to identify firms subject to earnings-based constraints. Facility-level syndicated loan terms used to build the sample of debtor-in-possession and highly speculative loans.</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>Proprietary</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr"/>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>syndicated loans; DIP; facilities; loan covenants; debt-to-EBITDA</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>Working Paper - 2026 - Dou et al. - The Cost of Intermediary Market Power for Distressed Borrowers; Working Paper - 2026 - Ebsim et al. - Sophisticated Borrowing Constraints and Macroeconomic Dynamics</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Robert Shiller</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Investor Confidence Survey</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr"/>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Investor-confidence survey data used as a comparison measure of investor beliefs.</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr"/>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>investor confidence; beliefs</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>Working Paper - 2026 - Thesmar and Verner - Beliefs and Stock Market Fluctuations New Evidence from the Past Seven Decades</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P Capital IQ</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr"/>
+      <c r="C36" s="2" t="inlineStr"/>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Supplementary financial data used to improve customer-capital expense measures.</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>Proprietary</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr"/>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>financials; customer capital</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>Working Paper - 2026 - Eisfeldt et al. - Intangible Intensity</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>SEC (WRDS SEC Analytics Suite)</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>10-K filings</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr"/>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Full-text corporate 10-K filings, accessed via the WRDS SEC Analytics Suite, used to build the text-based intangible-intensity measure.</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>Proprietary</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr"/>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>10-K; disclosure text; NLP</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>Working Paper - 2026 - Eisfeldt et al. - Intangible Intensity</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>U.S. Call Reports (via FOIA)</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr"/>
+      <c r="C38" s="2" t="inlineStr"/>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Bank-level regulatory balance-sheet data obtained back to 1959 through a Freedom of Information Act request, used to measure deposits and lending contractions.</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>Restricted</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr"/>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>call reports; bank lending; 1959-</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>Working Paper - 2026 - Drechsler et al. - Credit Crunches and the Great Stagflation</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>U.S. Census Bureau</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>LODES (LEHD Origin-Destination Employment Statistics)</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr"/>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>Sector-level job counts used to measure a city's industrial concentration.</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr"/>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>employment; industry concentration; LODES</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>Working Paper - 2026 - Ahern - Industrial Concentration, Property Values, and Municipal Bond Spreads</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>U.S. Census Bureau</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>LEHD merged with Longitudinal Business Database (LBD)</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr"/>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>Confidential administrative data on establishment-level wage bill and employment used to measure local monopsony power and firm responses to monetary policy.</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>Restricted</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr"/>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>administrative; wage bill; employment; monopsony</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>Working Paper - 2026 - Bardóczy et al. - Monopsony Power and the Transmission of Monetary Policy</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>U.S. Census Bureau</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>Longitudinal Business Database (LBD)</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr"/>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>Confidential data tracking entry and exit for the universe of U.S. employers, used to estimate the debt–exit relationship.</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>Restricted</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr"/>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>firm entry/exit; universe of employers</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I41" s="2" t="inlineStr">
+        <is>
+          <t>Working Paper - 2026 - Bornstein and Castillo-Martinez - Firm Exit and Financial Frictions</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>UBS/Gallup and Livingston Survey</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr"/>
+      <c r="C42" s="2" t="inlineStr"/>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Survey measures of individual-investor and professional-forecaster return/earnings expectations used for comparison.</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr"/>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>investor surveys; forecaster expectations</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>Working Paper - 2026 - Thesmar and Verner - Beliefs and Stock Market Fluctuations New Evidence from the Past Seven Decades</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>Value Line Investment Survey</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr"/>
+      <c r="C43" s="2" t="inlineStr"/>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>Analyst forecasts hand-collected from microfilm records (1956-2024) used to construct a long-run series of sophisticated investors' subjective expected returns.</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>Restricted</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr"/>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>subjective expectations; analyst forecasts; microfilm</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t>Working Paper - 2026 - Thesmar and Verner - Beliefs and Stock Market Fluctuations New Evidence from the Past Seven Decades</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>WIND</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr"/>
+      <c r="C44" s="2" t="inlineStr"/>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>Adjusted opening prices and free-floating shares for Chinese listed stocks.</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>Proprietary</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr"/>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
           <t>China; prices; shares</t>
         </is>
       </c>
-      <c r="H22" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="I22" s="2" t="inlineStr">
+      <c r="H44" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I44" s="2" t="inlineStr">
         <is>
           <t>Working Paper - 2026 - He et al. - Homemade Foreign Trading</t>
         </is>
       </c>
     </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>Yunan Ji</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>Medicare DME auction bids</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr"/>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>Bids submitted in Medicare's DME competitive-bidding auctions, shared by the author, used in the bidding analysis.</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>Restricted</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr"/>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>auction bids; competitive bidding</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I45" s="2" t="inlineStr">
+        <is>
+          <t>Working Paper - 2026 - Diwan et al. - Competition and Fraud in Health Care</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I22"/>
+  <autoFilter ref="A1:I45"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>